<commit_message>
Fixed normal commands. still need to do custom
</commit_message>
<xml_diff>
--- a/hw04/hw04/microcode.xlsx
+++ b/hw04/hw04/microcode.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huan\Documents\GT\Summer 2023\CS_2110\hw04\hw04\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bruh\Documents\GT\Summer 2023\CS_2110\hw04\hw04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB9E7A07-EAEA-47F1-A105-F0FE5CA3E72B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1D92551-0C40-45C2-846E-22BE8C6F3C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="microcode" sheetId="1" r:id="rId1"/>
@@ -25,8 +25,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -1123,14 +1121,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BW86"/>
-  <sheetFormatPr defaultColWidth="11.33203125" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="11.296875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="22.08203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="30" width="4.58203125" customWidth="1"/>
-    <col min="31" max="31" width="2.58203125" customWidth="1"/>
+    <col min="1" max="1" width="22.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="30" width="4.59765625" customWidth="1"/>
+    <col min="31" max="31" width="2.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:75" ht="88">
+    <row r="1" spans="1:75" ht="87">
       <c r="A1" s="41"/>
       <c r="B1" s="42"/>
       <c r="C1" s="55" t="s">
@@ -1254,7 +1252,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:75" ht="32.15" customHeight="1">
+    <row r="3" spans="1:75" ht="32.1" customHeight="1">
       <c r="A3" s="46" t="s">
         <v>23</v>
       </c>
@@ -1600,7 +1598,7 @@
         <v>2100038</v>
       </c>
     </row>
-    <row r="8" spans="1:75" ht="32.15" customHeight="1">
+    <row r="8" spans="1:75" ht="32.1" customHeight="1">
       <c r="A8" s="27" t="s">
         <v>27</v>
       </c>
@@ -1758,7 +1756,7 @@
         <v>0000020</v>
       </c>
     </row>
-    <row r="11" spans="1:75" ht="32.15" customHeight="1">
+    <row r="11" spans="1:75" ht="32.1" customHeight="1">
       <c r="A11" s="46" t="s">
         <v>28</v>
       </c>
@@ -1792,7 +1790,7 @@
       <c r="AC11" s="19"/>
       <c r="AD11" s="20"/>
     </row>
-    <row r="12" spans="1:75" ht="16" customHeight="1">
+    <row r="12" spans="1:75" ht="16.05" customHeight="1">
       <c r="A12" s="51"/>
       <c r="C12" s="62"/>
       <c r="D12" s="62"/>
@@ -1954,7 +1952,7 @@
       <c r="BV13" s="4"/>
       <c r="BW13" s="4"/>
     </row>
-    <row r="14" spans="1:75" ht="32.15" customHeight="1">
+    <row r="14" spans="1:75" ht="32.1" customHeight="1">
       <c r="A14" s="46" t="s">
         <v>30</v>
       </c>
@@ -2190,7 +2188,7 @@
         <v>188413F</v>
       </c>
     </row>
-    <row r="17" spans="1:34" ht="32.15" customHeight="1">
+    <row r="17" spans="1:34" ht="32.1" customHeight="1">
       <c r="A17" s="46" t="s">
         <v>32</v>
       </c>
@@ -2441,7 +2439,7 @@
         <v>041103F</v>
       </c>
     </row>
-    <row r="21" spans="1:34" ht="32.15" customHeight="1">
+    <row r="21" spans="1:34" ht="32.1" customHeight="1">
       <c r="A21" s="52" t="s">
         <v>35</v>
       </c>
@@ -2541,10 +2539,10 @@
         <v>0</v>
       </c>
       <c r="M23" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N23" s="30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O23" s="26">
         <v>0</v>
@@ -2556,19 +2554,19 @@
         <v>1</v>
       </c>
       <c r="R23" s="15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S23" s="30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T23" s="15">
         <v>0</v>
       </c>
       <c r="U23" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V23" s="30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W23" s="18">
         <v>0</v>
@@ -2596,10 +2594,10 @@
       </c>
       <c r="AH23" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C23:F23), 1), BIN2HEX(_xlfn.CONCAT(G23:N23), 2), BIN2HEX(_xlfn.CONCAT(O23:V23), 2), BIN2HEX(_xlfn.CONCAT(W23:AD23), 2) )</f>
-        <v>049783F</v>
-      </c>
-    </row>
-    <row r="24" spans="1:34" ht="32.15" customHeight="1">
+        <v>04A633F</v>
+      </c>
+    </row>
+    <row r="24" spans="1:34" ht="32.1" customHeight="1">
       <c r="A24" s="46" t="s">
         <v>37</v>
       </c>
@@ -2943,7 +2941,7 @@
         <v>161E03F</v>
       </c>
     </row>
-    <row r="29" spans="1:34" ht="32.15" customHeight="1">
+    <row r="29" spans="1:34" ht="32.1" customHeight="1">
       <c r="A29" s="46" t="s">
         <v>41</v>
       </c>
@@ -3287,7 +3285,7 @@
         <v>190003F</v>
       </c>
     </row>
-    <row r="34" spans="1:34" ht="32.15" customHeight="1">
+    <row r="34" spans="1:34" ht="32.1" customHeight="1">
       <c r="A34" s="46" t="s">
         <v>45</v>
       </c>
@@ -3817,7 +3815,7 @@
         <v>190003F</v>
       </c>
     </row>
-    <row r="41" spans="1:34" ht="32.15" customHeight="1">
+    <row r="41" spans="1:34" ht="32.1" customHeight="1">
       <c r="A41" s="46" t="s">
         <v>51</v>
       </c>
@@ -4161,7 +4159,7 @@
         <v>190003F</v>
       </c>
     </row>
-    <row r="46" spans="1:34" ht="32.15" customHeight="1">
+    <row r="46" spans="1:34" ht="32.1" customHeight="1">
       <c r="A46" s="46" t="s">
         <v>55</v>
       </c>
@@ -4276,10 +4274,10 @@
         <v>0</v>
       </c>
       <c r="R48" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S48" s="30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T48" s="15">
         <v>1</v>
@@ -4316,10 +4314,10 @@
       </c>
       <c r="AH48" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C48:F48), 1), BIN2HEX(_xlfn.CONCAT(G48:N48), 2), BIN2HEX(_xlfn.CONCAT(O48:V48), 2), BIN2HEX(_xlfn.CONCAT(W48:AD48), 2) )</f>
-        <v>1040C3F</v>
-      </c>
-    </row>
-    <row r="49" spans="1:34" ht="32.15" customHeight="1">
+        <v>104143F</v>
+      </c>
+    </row>
+    <row r="49" spans="1:34" ht="32.1" customHeight="1">
       <c r="A49" s="46" t="s">
         <v>57</v>
       </c>
@@ -4477,7 +4475,7 @@
         <v>188423F</v>
       </c>
     </row>
-    <row r="52" spans="1:34" ht="32.15" customHeight="1">
+    <row r="52" spans="1:34" ht="32.1" customHeight="1">
       <c r="A52" s="53" t="s">
         <v>59</v>
       </c>
@@ -4821,7 +4819,7 @@
         <v>00000FF</v>
       </c>
     </row>
-    <row r="57" spans="1:34" ht="32.15" customHeight="1">
+    <row r="57" spans="1:34" ht="32.1" customHeight="1">
       <c r="A57" s="53" t="s">
         <v>63</v>
       </c>
@@ -5165,7 +5163,7 @@
         <v>00000FF</v>
       </c>
     </row>
-    <row r="62" spans="1:34" ht="32.15" customHeight="1">
+    <row r="62" spans="1:34" ht="32.1" customHeight="1">
       <c r="A62" s="53" t="s">
         <v>67</v>
       </c>
@@ -5695,7 +5693,7 @@
         <v>00000FF</v>
       </c>
     </row>
-    <row r="69" spans="1:34" ht="32.15" customHeight="1">
+    <row r="69" spans="1:34" ht="32.1" customHeight="1">
       <c r="A69" s="46" t="s">
         <v>73</v>
       </c>
@@ -5853,7 +5851,7 @@
         <v>000000F</v>
       </c>
     </row>
-    <row r="72" spans="1:34" ht="31">
+    <row r="72" spans="1:34" ht="31.2">
       <c r="A72" s="27" t="s">
         <v>74</v>
       </c>
@@ -5887,7 +5885,7 @@
       <c r="AC72" s="19"/>
       <c r="AD72" s="20"/>
     </row>
-    <row r="73" spans="1:34" ht="31">
+    <row r="73" spans="1:34" ht="31.2">
       <c r="A73" s="28"/>
       <c r="B73" s="29"/>
       <c r="C73" s="11"/>
@@ -6028,7 +6026,7 @@
         <v>0</v>
       </c>
       <c r="F75" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G75" s="11">
         <v>1</v>
@@ -6104,7 +6102,7 @@
       </c>
       <c r="AH75" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C75:F75), 1), BIN2HEX(_xlfn.CONCAT(G75:N75), 2), BIN2HEX(_xlfn.CONCAT(O75:V75), 2), BIN2HEX(_xlfn.CONCAT(W75:AD75), 2) )</f>
-        <v>8842C1F</v>
+        <v>9842C1F</v>
       </c>
     </row>
     <row r="76" spans="1:34">
@@ -6213,10 +6211,10 @@
         <v>0</v>
       </c>
       <c r="E77" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F77" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G77" s="11">
         <v>0</v>
@@ -6270,7 +6268,7 @@
         <v>1</v>
       </c>
       <c r="X77" s="69">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y77" s="31">
         <v>1</v>
@@ -6292,7 +6290,7 @@
       </c>
       <c r="AH77" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C77:F77), 1), BIN2HEX(_xlfn.CONCAT(G77:N77), 2), BIN2HEX(_xlfn.CONCAT(O77:V77), 2), BIN2HEX(_xlfn.CONCAT(W77:AD77), 2) )</f>
-        <v>00000FF</v>
+        <v>30000BF</v>
       </c>
     </row>
     <row r="78" spans="1:34">
@@ -6327,7 +6325,7 @@
       <c r="AC78" s="31"/>
       <c r="AD78" s="21"/>
     </row>
-    <row r="79" spans="1:34" ht="31">
+    <row r="79" spans="1:34" ht="31.2">
       <c r="A79" s="27" t="s">
         <v>79</v>
       </c>
@@ -6361,7 +6359,7 @@
       <c r="AC79" s="19"/>
       <c r="AD79" s="20"/>
     </row>
-    <row r="80" spans="1:34" ht="31">
+    <row r="80" spans="1:34" ht="31.2">
       <c r="A80" s="28"/>
       <c r="B80" s="29"/>
       <c r="C80" s="11"/>
@@ -6514,7 +6512,7 @@
         <v>0</v>
       </c>
       <c r="J82" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K82" s="13">
         <v>0</v>
@@ -6578,7 +6576,7 @@
       </c>
       <c r="AH82" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C82:F82), 1), BIN2HEX(_xlfn.CONCAT(G82:N82), 2), BIN2HEX(_xlfn.CONCAT(O82:V82), 2), BIN2HEX(_xlfn.CONCAT(W82:AD82), 2) )</f>
-        <v>4100095</v>
+        <v>4000095</v>
       </c>
     </row>
     <row r="83" spans="1:36">
@@ -6702,7 +6700,7 @@
         <v>0</v>
       </c>
       <c r="J84" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K84" s="13">
         <v>0</v>
@@ -6766,7 +6764,7 @@
       </c>
       <c r="AH84" t="str">
         <f t="shared" ref="AH84:AH85" si="4">_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C84:F84), 1), BIN2HEX(_xlfn.CONCAT(G84:N84), 2), BIN2HEX(_xlfn.CONCAT(O84:V84), 2), BIN2HEX(_xlfn.CONCAT(W84:AD84), 2) )</f>
-        <v>410009C</v>
+        <v>400009C</v>
       </c>
       <c r="AI84" s="5"/>
       <c r="AJ84" s="5"/>
@@ -6798,19 +6796,19 @@
         <v>0</v>
       </c>
       <c r="J85" s="13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K85" s="13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L85" s="13">
         <v>0</v>
       </c>
       <c r="M85" s="15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N85" s="30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O85" s="26">
         <v>0</v>
@@ -6819,7 +6817,7 @@
         <v>0</v>
       </c>
       <c r="Q85" s="30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R85" s="15">
         <v>0</v>
@@ -6862,7 +6860,7 @@
       </c>
       <c r="AH85" t="str">
         <f t="shared" si="4"/>
-        <v>04A003F</v>
+        <v>051203F</v>
       </c>
       <c r="AI85" s="5"/>
       <c r="AJ85" s="5"/>
@@ -6909,10 +6907,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F64"/>
-  <sheetFormatPr defaultColWidth="11.08203125" defaultRowHeight="15.5"/>
+  <sheetFormatPr defaultColWidth="11.09765625" defaultRowHeight="15.6"/>
   <cols>
     <col min="3" max="3" width="15.5" customWidth="1"/>
-    <col min="6" max="6" width="10.58203125" customWidth="1"/>
+    <col min="6" max="6" width="10.59765625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -7123,7 +7121,7 @@
       </c>
       <c r="D13" s="6" t="str">
         <f>microcode!AH23</f>
-        <v>049783F</v>
+        <v>04A633F</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -7155,7 +7153,7 @@
       </c>
       <c r="D15" s="6" t="str">
         <f>microcode!AH48</f>
-        <v>1040C3F</v>
+        <v>104143F</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -7203,7 +7201,7 @@
       </c>
       <c r="D18" s="6" t="str">
         <f>microcode!AH82</f>
-        <v>4100095</v>
+        <v>4000095</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -7238,7 +7236,7 @@
         <v>4080323</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="17">
+    <row r="21" spans="1:5" ht="17.399999999999999">
       <c r="A21" s="5">
         <v>20</v>
       </c>
@@ -7332,7 +7330,7 @@
       </c>
       <c r="D26" s="6" t="str">
         <f>microcode!AH84</f>
-        <v>410009C</v>
+        <v>400009C</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -7380,7 +7378,7 @@
       </c>
       <c r="D29" s="6" t="str">
         <f>microcode!AH85</f>
-        <v>04A003F</v>
+        <v>051203F</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -7412,7 +7410,7 @@
       </c>
       <c r="D31" s="6" t="str">
         <f>microcode!AH75</f>
-        <v>8842C1F</v>
+        <v>9842C1F</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -7459,7 +7457,7 @@
       </c>
       <c r="D34" s="6" t="str">
         <f>microcode!AH77</f>
-        <v>00000FF</v>
+        <v>30000BF</v>
       </c>
     </row>
     <row r="35" spans="1:4">

</xml_diff>